<commit_message>
Translate comments, add gene sets and figure inputs
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplementary_tables/Supplementary_Table_S1.xlsx
+++ b/supplementary_tables/Supplementary_Table_S1.xlsx
@@ -66,7 +66,7 @@
     <t xml:space="preserve">OS</t>
   </si>
   <si>
-    <t xml:space="preserve">正文公式(Results/Methods段)</t>
+    <t xml:space="preserve">Risk-score formula in main text (Results/Methods)</t>
   </si>
   <si>
     <t xml:space="preserve">S002</t>
@@ -264,7 +264,7 @@
     <t xml:space="preserve">Front Oncol</t>
   </si>
   <si>
-    <t xml:space="preserve">正文公式(人工抄录)</t>
+    <t xml:space="preserve">Risk-score formula in main text (manually transcribed)</t>
   </si>
   <si>
     <t xml:space="preserve">S019</t>

</xml_diff>